<commit_message>
Add ML iteration results: 10 iterations completed
</commit_message>
<xml_diff>
--- a/output/ml_iterations_all_results_10.xlsx
+++ b/output/ml_iterations_all_results_10.xlsx
@@ -545,13 +545,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9943512612719275</v>
+        <v>0.9654915102563981</v>
       </c>
       <c r="C2" t="n">
-        <v>0.534285865860741</v>
+        <v>1.422892857142855</v>
       </c>
       <c r="D2" t="n">
-        <v>1.343826781038538</v>
+        <v>3.598811744856232</v>
       </c>
       <c r="E2" t="n">
         <v>0.9951717259446977</v>
@@ -563,31 +563,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H2" t="n">
-        <v>-6.997949856618484</v>
+        <v>-65.16871150409727</v>
       </c>
       <c r="I2" t="n">
-        <v>0.009681547619048214</v>
+        <v>0.01132046341793541</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5018336666413123</v>
+        <v>0.585014958470643</v>
       </c>
       <c r="K2" t="n">
-        <v>-11.12275366268994</v>
+        <v>-8.77566551959119</v>
       </c>
       <c r="L2" t="n">
-        <v>0.009044285714286338</v>
+        <v>0.008503472222223141</v>
       </c>
       <c r="M2" t="n">
-        <v>0.4933193002254272</v>
+        <v>0.4641083438655683</v>
       </c>
       <c r="N2" t="n">
-        <v>0.04042268953363237</v>
+        <v>-0.04892835665438344</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3913678571428573</v>
+        <v>0.3933875000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>38.35905299672125</v>
+        <v>38.02740147867898</v>
       </c>
       <c r="Q2" t="n">
         <v>0.7713865597315819</v>
@@ -613,13 +613,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9838047263944724</v>
+        <v>0.9879559468969878</v>
       </c>
       <c r="C3" t="n">
-        <v>1.024916666666668</v>
+        <v>0.9175416666666667</v>
       </c>
       <c r="D3" t="n">
-        <v>2.651645518216498</v>
+        <v>2.404231163553595</v>
       </c>
       <c r="E3" t="n">
         <v>0.9951717259446977</v>
@@ -631,31 +631,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H3" t="n">
-        <v>-65.16871150409727</v>
+        <v>-6.862421982154753</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01132046341793541</v>
+        <v>0.009563888888888761</v>
       </c>
       <c r="J3" t="n">
-        <v>0.585014958470643</v>
+        <v>0.4958729169375468</v>
       </c>
       <c r="K3" t="n">
-        <v>-9.306005321799727</v>
+        <v>-9.596258661600464</v>
       </c>
       <c r="L3" t="n">
-        <v>0.008639523809524985</v>
+        <v>0.008782110389610964</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4715488262924946</v>
+        <v>0.4791989471346915</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2204746352714769</v>
+        <v>-0.07369858079878311</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3748294642857145</v>
+        <v>0.3959833333333334</v>
       </c>
       <c r="P3" t="n">
-        <v>38.34408991501635</v>
+        <v>38.03518129044393</v>
       </c>
       <c r="Q3" t="n">
         <v>0.7713865597315819</v>
@@ -681,13 +681,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.9943512612719275</v>
+        <v>0.9782843614770297</v>
       </c>
       <c r="C4" t="n">
-        <v>0.534285865860741</v>
+        <v>1.08127976190476</v>
       </c>
       <c r="D4" t="n">
-        <v>1.343826781038538</v>
+        <v>2.830821354798675</v>
       </c>
       <c r="E4" t="n">
         <v>0.9951717259446977</v>
@@ -699,31 +699,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H4" t="n">
-        <v>-8.67713885903081</v>
+        <v>-9.658662479064489</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01085351190476225</v>
+        <v>0.01027273809523838</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5624179689457269</v>
+        <v>0.5324210495325946</v>
       </c>
       <c r="K4" t="n">
-        <v>-10.34759227759577</v>
+        <v>-14.22281816386041</v>
       </c>
       <c r="L4" t="n">
-        <v>0.008214345238095666</v>
+        <v>0.008347023809524734</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4482975068275623</v>
+        <v>0.4553929197975934</v>
       </c>
       <c r="N4" t="n">
-        <v>0.07928525078312687</v>
+        <v>-0.07928640487822469</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3902755952380952</v>
+        <v>0.4059375000000002</v>
       </c>
       <c r="P4" t="n">
-        <v>37.85749862095661</v>
+        <v>38.07976433698515</v>
       </c>
       <c r="Q4" t="n">
         <v>0.7713865597315819</v>
@@ -749,13 +749,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.9835607461227431</v>
+        <v>0.9943512612719275</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9063095238095249</v>
+        <v>0.534285865860741</v>
       </c>
       <c r="D5" t="n">
-        <v>2.267432864317044</v>
+        <v>1.343826781038538</v>
       </c>
       <c r="E5" t="n">
         <v>0.9951717259446977</v>
@@ -767,31 +767,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H5" t="n">
-        <v>-65.16871150409727</v>
+        <v>-5.936848880562593</v>
       </c>
       <c r="I5" t="n">
-        <v>0.01132046341793541</v>
+        <v>0.009385654761905227</v>
       </c>
       <c r="J5" t="n">
-        <v>0.585014958470643</v>
+        <v>0.4868036738758381</v>
       </c>
       <c r="K5" t="n">
-        <v>-8.684614040037394</v>
+        <v>-10.67230413928855</v>
       </c>
       <c r="L5" t="n">
-        <v>0.007639464285714992</v>
+        <v>0.009385357142858264</v>
       </c>
       <c r="M5" t="n">
-        <v>0.417093981576137</v>
+        <v>0.5119128840307403</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1636364425552007</v>
+        <v>0.06859589901496665</v>
       </c>
       <c r="O5" t="n">
-        <v>0.3853333333333333</v>
+        <v>0.4052458333333333</v>
       </c>
       <c r="P5" t="n">
-        <v>38.2586174207322</v>
+        <v>39.06669075940758</v>
       </c>
       <c r="Q5" t="n">
         <v>0.7713865597315819</v>
@@ -817,13 +817,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.9757594314420815</v>
+        <v>0.9881121096661553</v>
       </c>
       <c r="C6" t="n">
-        <v>1.137404761904767</v>
+        <v>0.802782738095237</v>
       </c>
       <c r="D6" t="n">
-        <v>2.913371050238949</v>
+        <v>2.081661143104006</v>
       </c>
       <c r="E6" t="n">
         <v>0.9951717259446977</v>
@@ -835,31 +835,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H6" t="n">
-        <v>-65.16871150409727</v>
+        <v>-12.65831552181593</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01132046341793541</v>
+        <v>0.0104091170634919</v>
       </c>
       <c r="J6" t="n">
-        <v>0.585014958470643</v>
+        <v>0.5392151002418375</v>
       </c>
       <c r="K6" t="n">
-        <v>-11.07236607180633</v>
+        <v>-8.024484841361247</v>
       </c>
       <c r="L6" t="n">
-        <v>0.008750744047619996</v>
+        <v>0.008410625000000949</v>
       </c>
       <c r="M6" t="n">
-        <v>0.477346443019338</v>
+        <v>0.458996855384928</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1074815004558106</v>
+        <v>0.09501934763706044</v>
       </c>
       <c r="O6" t="n">
-        <v>0.3782583333333334</v>
+        <v>0.400179166666666</v>
       </c>
       <c r="P6" t="n">
-        <v>37.77325850598061</v>
+        <v>40.51347507252702</v>
       </c>
       <c r="Q6" t="n">
         <v>0.7713865597315819</v>
@@ -885,13 +885,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.9861041590228216</v>
+        <v>0.9764685471558699</v>
       </c>
       <c r="C7" t="n">
-        <v>1.006458333333327</v>
+        <v>1.141505952380959</v>
       </c>
       <c r="D7" t="n">
-        <v>2.546330544582312</v>
+        <v>2.866984804342379</v>
       </c>
       <c r="E7" t="n">
         <v>0.9951717259446977</v>
@@ -903,31 +903,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H7" t="n">
-        <v>-65.16871150409727</v>
+        <v>-6.054635639196762</v>
       </c>
       <c r="I7" t="n">
-        <v>0.01132046341793541</v>
+        <v>0.009211458333333811</v>
       </c>
       <c r="J7" t="n">
-        <v>0.585014958470643</v>
+        <v>0.4777346480100177</v>
       </c>
       <c r="K7" t="n">
-        <v>-10.26553913155825</v>
+        <v>-7.957610982155892</v>
       </c>
       <c r="L7" t="n">
-        <v>0.008703988095238313</v>
+        <v>0.008804880952381577</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4749552212763916</v>
+        <v>0.4803698319854957</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.03133474500563138</v>
+        <v>0.01656595502141667</v>
       </c>
       <c r="O7" t="n">
-        <v>0.394109920634921</v>
+        <v>0.3972523809523805</v>
       </c>
       <c r="P7" t="n">
-        <v>37.85852659553261</v>
+        <v>39.24930860252469</v>
       </c>
       <c r="Q7" t="n">
         <v>0.7713865597315819</v>
@@ -980,22 +980,22 @@
         <v>0.585014958470643</v>
       </c>
       <c r="K8" t="n">
-        <v>-17.36186754408596</v>
+        <v>-12.21825959961859</v>
       </c>
       <c r="L8" t="n">
-        <v>0.008418958333334559</v>
+        <v>0.008704702380953555</v>
       </c>
       <c r="M8" t="n">
-        <v>0.4592447669274054</v>
+        <v>0.4749524930243599</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.077831014812352</v>
+        <v>0.236057855384601</v>
       </c>
       <c r="O8" t="n">
-        <v>0.4072875000000001</v>
+        <v>0.3620291666666667</v>
       </c>
       <c r="P8" t="n">
-        <v>38.61653244178205</v>
+        <v>37.28939688115593</v>
       </c>
       <c r="Q8" t="n">
         <v>0.7713865597315819</v>
@@ -1021,13 +1021,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.9795152274476511</v>
+        <v>0.9714822725572724</v>
       </c>
       <c r="C9" t="n">
-        <v>1.125625000000002</v>
+        <v>1.088080357142858</v>
       </c>
       <c r="D9" t="n">
-        <v>2.868920546542478</v>
+        <v>2.942744877730754</v>
       </c>
       <c r="E9" t="n">
         <v>0.9951717259446977</v>
@@ -1039,31 +1039,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H9" t="n">
-        <v>-5.54579595505641</v>
+        <v>-65.16871150409727</v>
       </c>
       <c r="I9" t="n">
-        <v>0.009544255952381342</v>
+        <v>0.01132046341793541</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4950027954200577</v>
+        <v>0.585014958470643</v>
       </c>
       <c r="K9" t="n">
-        <v>-7.669636604370124</v>
+        <v>-11.00517117943549</v>
       </c>
       <c r="L9" t="n">
-        <v>0.008893869047620129</v>
+        <v>0.009008392857143777</v>
       </c>
       <c r="M9" t="n">
-        <v>0.485400557198909</v>
+        <v>0.4913780567759304</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1463311260445673</v>
+        <v>-0.2481152670196873</v>
       </c>
       <c r="O9" t="n">
-        <v>0.3851708333333331</v>
+        <v>0.4062791666666659</v>
       </c>
       <c r="P9" t="n">
-        <v>37.96878115921582</v>
+        <v>37.81897683049086</v>
       </c>
       <c r="Q9" t="n">
         <v>0.7713865597315819</v>
@@ -1116,22 +1116,22 @@
         <v>0.585014958470643</v>
       </c>
       <c r="K10" t="n">
-        <v>-9.264405172992401</v>
+        <v>-12.59400833983281</v>
       </c>
       <c r="L10" t="n">
-        <v>0.009462767857143728</v>
+        <v>0.008545684523810271</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5160991966592267</v>
+        <v>0.46614661045552</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2385764837500183</v>
+        <v>0.1678659396026995</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3622613095238095</v>
+        <v>0.3777250000000004</v>
       </c>
       <c r="P10" t="n">
-        <v>38.10048594544398</v>
+        <v>38.09941110345504</v>
       </c>
       <c r="Q10" t="n">
         <v>0.7713865597315819</v>
@@ -1157,13 +1157,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.980948323477176</v>
+        <v>0.9768017793384227</v>
       </c>
       <c r="C11" t="n">
-        <v>1.108470238095235</v>
+        <v>1.167208333333334</v>
       </c>
       <c r="D11" t="n">
-        <v>2.877650781350012</v>
+        <v>3.037379147545608</v>
       </c>
       <c r="E11" t="n">
         <v>0.9951717259446977</v>
@@ -1175,31 +1175,31 @@
         <v>1.63170262213994</v>
       </c>
       <c r="H11" t="n">
-        <v>-9.488323126966625</v>
+        <v>-65.16871150409727</v>
       </c>
       <c r="I11" t="n">
-        <v>0.01094059523809537</v>
+        <v>0.01132046341793541</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5667240734358375</v>
+        <v>0.585014958470643</v>
       </c>
       <c r="K11" t="n">
-        <v>-8.4454926618131</v>
+        <v>-11.31480007074298</v>
       </c>
       <c r="L11" t="n">
-        <v>0.009270535714286821</v>
+        <v>0.008418452380953567</v>
       </c>
       <c r="M11" t="n">
-        <v>0.5057259090015473</v>
+        <v>0.4593635784870452</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.1107570766433568</v>
+        <v>0.05136518139827073</v>
       </c>
       <c r="O11" t="n">
-        <v>0.4077416666666669</v>
+        <v>0.3974180555555554</v>
       </c>
       <c r="P11" t="n">
-        <v>38.19139969730802</v>
+        <v>38.26233978634282</v>
       </c>
       <c r="Q11" t="n">
         <v>0.7713865597315819</v>

</xml_diff>